<commit_message>
create new annuities in annuities_certain.py
</commit_message>
<xml_diff>
--- a/soa_tables/tables_manual.xlsx
+++ b/soa_tables/tables_manual.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10520"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10814"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrocortereal/Dropbox (MagentaKoncept)/PedroCR/PycharmProjects/lifeActuary/soa_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC40A0D-93F4-3A4A-B1D6-FAB2B34F4916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E200DF3-5F4C-CB46-9EA8-5ADA0692CE94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16620" activeTab="1" xr2:uid="{BD97DD2D-0F63-8D44-8A57-7FC915C77CD0}"/>
+    <workbookView xWindow="2600" yWindow="760" windowWidth="27640" windowHeight="16620" xr2:uid="{BD97DD2D-0F63-8D44-8A57-7FC915C77CD0}"/>
   </bookViews>
   <sheets>
     <sheet name="qx" sheetId="1" r:id="rId1"/>
     <sheet name="lx" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
   <si>
     <t>TV7377</t>
   </si>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>GRM95</t>
+  </si>
+  <si>
+    <t>S2PMA</t>
+  </si>
+  <si>
+    <t>S2PFA</t>
   </si>
 </sst>
 </file>
@@ -397,10 +403,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26137DBD-82FB-7943-99FE-9F7E68E8EFF3}">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -410,8 +419,14 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
@@ -421,8 +436,14 @@
       <c r="C2">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1.1679999999999999E-2</v>
       </c>
@@ -432,8 +453,14 @@
       <c r="C3">
         <v>1.2879E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>9.7134529999999997E-4</v>
       </c>
@@ -443,8 +470,14 @@
       <c r="C4">
         <v>1.289E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>5.9755310000000005E-4</v>
       </c>
@@ -454,8 +487,14 @@
       <c r="C5">
         <v>1.2902E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4.661674E-4</v>
       </c>
@@ -465,8 +504,14 @@
       <c r="C6">
         <v>1.2913E-3</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3.8527439999999999E-4</v>
       </c>
@@ -476,8 +521,14 @@
       <c r="C7">
         <v>1.2924E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3.4485210000000002E-4</v>
       </c>
@@ -487,8 +538,14 @@
       <c r="C8">
         <v>1.2936E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>3.1453239999999999E-4</v>
       </c>
@@ -498,8 +555,14 @@
       <c r="C9">
         <v>1.2947E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2.943326E-4</v>
       </c>
@@ -509,8 +572,14 @@
       <c r="C10">
         <v>1.2957999999999999E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2.7411450000000001E-4</v>
       </c>
@@ -520,8 +589,14 @@
       <c r="C11">
         <v>1.297E-3</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2.5387929999999998E-4</v>
       </c>
@@ -531,8 +606,14 @@
       <c r="C12">
         <v>1.2980999999999999E-3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2.3362820000000001E-4</v>
       </c>
@@ -542,8 +623,14 @@
       <c r="C13">
         <v>1.2991999999999999E-3</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2.336828E-4</v>
       </c>
@@ -553,8 +640,14 @@
       <c r="C14">
         <v>1.3004E-3</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2.23575E-4</v>
       </c>
@@ -564,8 +657,14 @@
       <c r="C15">
         <v>1.3014999999999999E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2.5411930000000002E-4</v>
       </c>
@@ -575,8 +674,14 @@
       <c r="C16">
         <v>1.3025999999999999E-3</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>3.0502060000000002E-4</v>
       </c>
@@ -586,8 +691,14 @@
       <c r="C17">
         <v>1.3037999999999999E-3</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>3.8647740000000001E-4</v>
       </c>
@@ -597,8 +708,14 @@
       <c r="C18">
         <v>1.3056999999999999E-3</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>4.7819630000000001E-4</v>
       </c>
@@ -608,8 +725,14 @@
       <c r="C19">
         <v>1.3146E-3</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <v>3.0299999999999999E-4</v>
+      </c>
+      <c r="E19">
+        <v>1.7100000000000001E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>5.8021760000000005E-4</v>
       </c>
@@ -619,8 +742,14 @@
       <c r="C20">
         <v>1.3324999999999999E-3</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <v>3.1000393119118351E-4</v>
+      </c>
+      <c r="E20">
+        <v>1.7499992498714486E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>6.4166549999999998E-4</v>
       </c>
@@ -630,8 +759,14 @@
       <c r="C21">
         <v>1.3596000000000001E-3</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <v>3.1799490225547155E-4</v>
+      </c>
+      <c r="E21">
+        <v>1.8100262147701293E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>6.5226919999999999E-4</v>
       </c>
@@ -641,8 +776,14 @@
       <c r="C22">
         <v>1.3965E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D22">
+        <v>3.270043462151357E-4</v>
+      </c>
+      <c r="E22">
+        <v>1.8699853139620125E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>6.3229819999999996E-4</v>
       </c>
@@ -652,8 +793,14 @@
       <c r="C23">
         <v>1.4436E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D23">
+        <v>3.359924803046086E-4</v>
+      </c>
+      <c r="E23">
+        <v>1.9399847805360549E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>6.2249340000000003E-4</v>
       </c>
@@ -663,8 +810,14 @@
       <c r="C24">
         <v>1.5014E-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D24">
+        <v>3.470027684701875E-4</v>
+      </c>
+      <c r="E24">
+        <v>2.0300426087741939E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>6.024588E-4</v>
       </c>
@@ -674,8 +827,14 @@
       <c r="C25">
         <v>1.5709999999999999E-3</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D25">
+        <v>3.5900626752536621E-4</v>
+      </c>
+      <c r="E25">
+        <v>2.1299653051718334E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>5.9260469999999996E-4</v>
       </c>
@@ -685,8 +844,14 @@
       <c r="C26">
         <v>1.6535E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D26">
+        <v>3.7399935327400577E-4</v>
+      </c>
+      <c r="E26">
+        <v>2.2599905324716273E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>6.1340289999999996E-4</v>
       </c>
@@ -696,8 +861,14 @@
       <c r="C27">
         <v>1.7501000000000001E-3</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D27">
+        <v>3.8899896956780201E-4</v>
+      </c>
+      <c r="E27">
+        <v>2.4000175071176965E-4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>6.0354970000000001E-4</v>
       </c>
@@ -707,8 +878,14 @@
       <c r="C28">
         <v>1.8617E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <v>4.0699493237895804E-4</v>
+      </c>
+      <c r="E28">
+        <v>2.5599787267514655E-4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>6.1415000000000005E-4</v>
       </c>
@@ -718,8 +895,14 @@
       <c r="C29">
         <v>1.9895999999999998E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D29">
+        <v>4.2699937777426153E-4</v>
+      </c>
+      <c r="E29">
+        <v>2.7600418567608475E-4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>6.2476960000000005E-4</v>
       </c>
@@ -729,8 +912,14 @@
       <c r="C30">
         <v>2.1348000000000001E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D30">
+        <v>4.4800278009488422E-4</v>
+      </c>
+      <c r="E30">
+        <v>2.980012317370274E-4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>6.7640280000000005E-4</v>
       </c>
@@ -740,8 +929,14 @@
       <c r="C31">
         <v>2.2989999999999998E-3</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D31">
+        <v>4.7300110781384414E-4</v>
+      </c>
+      <c r="E31">
+        <v>3.2299523654467997E-4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>7.1788250000000004E-4</v>
       </c>
@@ -751,8 +946,14 @@
       <c r="C32">
         <v>2.4854999999999999E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>5.0000367767987712E-4</v>
+      </c>
+      <c r="E32">
+        <v>3.5200454840783368E-4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>7.389238E-4</v>
       </c>
@@ -762,8 +963,14 @@
       <c r="C33">
         <v>2.6984000000000001E-3</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>5.2999156284148387E-4</v>
+      </c>
+      <c r="E33">
+        <v>3.8499663507942636E-4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>7.9082239999999997E-4</v>
       </c>
@@ -773,8 +980,14 @@
       <c r="C34">
         <v>2.9413999999999998E-3</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>5.6300349266957025E-4</v>
+      </c>
+      <c r="E34">
+        <v>4.230039982485154E-4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>8.4284099999999999E-4</v>
       </c>
@@ -784,8 +997,14 @@
       <c r="C35">
         <v>3.2187000000000001E-3</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>6.0100149336535507E-4</v>
+      </c>
+      <c r="E35">
+        <v>4.6599834243194447E-4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>9.0527529999999998E-4</v>
       </c>
@@ -795,8 +1014,14 @@
       <c r="C36">
         <v>3.5338000000000001E-3</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <v>6.4199690351876386E-4</v>
+      </c>
+      <c r="E36">
+        <v>5.1399342968424546E-4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>9.781713E-4</v>
       </c>
@@ -806,8 +1031,14 @@
       <c r="C37">
         <v>3.8714999999999999E-3</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <v>6.8799700225774865E-4</v>
+      </c>
+      <c r="E37">
+        <v>5.6800027829118495E-4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>1.0615821E-3</v>
       </c>
@@ -817,8 +1048,14 @@
       <c r="C38">
         <v>4.2176000000000002E-3</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>7.3900053278704145E-4</v>
+      </c>
+      <c r="E38">
+        <v>6.2900509156618256E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>1.1349331999999999E-3</v>
       </c>
@@ -828,8 +1065,14 @@
       <c r="C39">
         <v>4.5777999999999999E-3</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>7.9500854678091291E-4</v>
+      </c>
+      <c r="E39">
+        <v>6.9599798441947666E-4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1.2498450999999999E-3</v>
       </c>
@@ -839,8 +1082,14 @@
       <c r="C40">
         <v>4.9576000000000004E-3</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>8.5699418427180596E-4</v>
+      </c>
+      <c r="E40">
+        <v>7.7100086927419037E-4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1.3444891E-3</v>
       </c>
@@ -850,8 +1099,14 @@
       <c r="C41">
         <v>5.3626000000000004E-3</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>9.2499757738007267E-4</v>
+      </c>
+      <c r="E41">
+        <v>8.5400184381199333E-4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1.470573E-3</v>
       </c>
@@ -861,8 +1116,14 @@
       <c r="C42">
         <v>5.7984999999999998E-3</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D42">
+        <v>1.0000036523438831E-3</v>
+      </c>
+      <c r="E42">
+        <v>9.4599355103691901E-4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1.6179384000000001E-3</v>
       </c>
@@ -872,8 +1133,14 @@
       <c r="C43">
         <v>6.2708E-3</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D43">
+        <v>1.0829962808657741E-3</v>
+      </c>
+      <c r="E43">
+        <v>1.0460012692834143E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1.755607E-3</v>
       </c>
@@ -883,8 +1150,14 @@
       <c r="C44">
         <v>6.7850999999999996E-3</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D44">
+        <v>1.173003123104711E-3</v>
+      </c>
+      <c r="E44">
+        <v>1.156004437047001E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1.9147917999999999E-3</v>
       </c>
@@ -894,8 +1167,14 @@
       <c r="C45">
         <v>7.3470000000000002E-3</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D45">
+        <v>1.2730010837891854E-3</v>
+      </c>
+      <c r="E45">
+        <v>1.2749970012124088E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2.1165676E-3</v>
       </c>
@@ -905,8 +1184,14 @@
       <c r="C46">
         <v>7.9620999999999997E-3</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D46">
+        <v>1.383004552108297E-3</v>
+      </c>
+      <c r="E46">
+        <v>1.4040034913927202E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2.3195796000000002E-3</v>
       </c>
@@ -916,8 +1201,14 @@
       <c r="C47">
         <v>8.6361000000000007E-3</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D47">
+        <v>1.5019998235660085E-3</v>
+      </c>
+      <c r="E47">
+        <v>1.5439952668951712E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2.5134837999999998E-3</v>
       </c>
@@ -927,8 +1218,14 @@
       <c r="C48">
         <v>9.3743999999999997E-3</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D48">
+        <v>1.6329921638534965E-3</v>
+      </c>
+      <c r="E48">
+        <v>1.693007125704935E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2.7508006000000001E-3</v>
       </c>
@@ -938,8 +1235,14 @@
       <c r="C49">
         <v>1.0182800000000001E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D49">
+        <v>1.7770007907717826E-3</v>
+      </c>
+      <c r="E49">
+        <v>1.8539981920076367E-3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>3.0005369000000001E-3</v>
       </c>
@@ -949,8 +1252,14 @@
       <c r="C50">
         <v>1.10668E-2</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D50">
+        <v>1.933003575577467E-3</v>
+      </c>
+      <c r="E50">
+        <v>2.0249922154512612E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>3.2735644000000002E-3</v>
       </c>
@@ -960,8 +1269,14 @@
       <c r="C51">
         <v>1.19579E-2</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D51">
+        <v>2.1029992843090459E-3</v>
+      </c>
+      <c r="E51">
+        <v>2.2060036228788321E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>3.5173963E-3</v>
       </c>
@@ -971,8 +1286,14 @@
       <c r="C52">
         <v>1.2818100000000001E-2</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D52">
+        <v>2.2900016552410509E-3</v>
+      </c>
+      <c r="E52">
+        <v>2.398998635731231E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>3.7637152E-3</v>
       </c>
@@ -982,8 +1303,14 @@
       <c r="C53">
         <v>1.3696699999999999E-2</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D53">
+        <v>2.4939947406603389E-3</v>
+      </c>
+      <c r="E53">
+        <v>2.6010058930901491E-3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4.0554097000000001E-3</v>
       </c>
@@ -993,8 +1320,14 @@
       <c r="C54">
         <v>1.464E-2</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D54">
+        <v>2.7170050453446787E-3</v>
+      </c>
+      <c r="E54">
+        <v>2.8129986675713356E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4.4148217999999996E-3</v>
       </c>
@@ -1004,8 +1337,14 @@
       <c r="C55">
         <v>1.5691299999999998E-2</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D55">
+        <v>2.960002772807298E-3</v>
+      </c>
+      <c r="E55">
+        <v>3.0329978532697591E-3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4.7895812999999999E-3</v>
       </c>
@@ -1015,8 +1354,14 @@
       <c r="C56">
         <v>1.6891199999999999E-2</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D56">
+        <v>3.2249988188366029E-3</v>
+      </c>
+      <c r="E56">
+        <v>3.2620045954554248E-3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>5.1695235999999999E-3</v>
       </c>
@@ -1026,8 +1371,14 @@
       <c r="C57">
         <v>1.8277600000000001E-2</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D57">
+        <v>3.5120007090858104E-3</v>
+      </c>
+      <c r="E57">
+        <v>3.4969907761643634E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>5.5333906000000002E-3</v>
       </c>
@@ -1037,8 +1388,14 @@
       <c r="C58">
         <v>1.98861E-2</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D58">
+        <v>3.822992836563534E-3</v>
+      </c>
+      <c r="E58">
+        <v>3.7390089828810507E-3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>5.9030586999999999E-3</v>
       </c>
@@ -1048,8 +1405,14 @@
       <c r="C59">
         <v>2.1749600000000001E-2</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D59">
+        <v>4.1590076968171215E-3</v>
+      </c>
+      <c r="E59">
+        <v>3.9839954726520761E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>6.3119928E-3</v>
       </c>
@@ -1059,8 +1422,14 @@
       <c r="C60">
         <v>2.3889199999999999E-2</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D60">
+        <v>4.5230001783979979E-3</v>
+      </c>
+      <c r="E60">
+        <v>4.232995720788447E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>6.7504758999999996E-3</v>
       </c>
@@ -1070,8 +1439,14 @@
       <c r="C61">
         <v>2.6286299999999999E-2</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D61">
+        <v>4.9149905561636006E-3</v>
+      </c>
+      <c r="E61">
+        <v>4.4840011618272639E-3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>7.2197338999999998E-3</v>
       </c>
@@ -1081,8 +1456,14 @@
       <c r="C62">
         <v>2.8913899999999999E-2</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D62">
+        <v>5.3380034378338543E-3</v>
+      </c>
+      <c r="E62">
+        <v>4.7350056353599665E-3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>7.7323636999999997E-3</v>
       </c>
@@ -1092,8 +1473,14 @@
       <c r="C63">
         <v>3.1746200000000002E-2</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D63">
+        <v>5.7970053472941353E-3</v>
+      </c>
+      <c r="E63">
+        <v>4.9909926404774312E-3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>8.4033613000000004E-3</v>
       </c>
@@ -1103,8 +1490,14 @@
       <c r="C64">
         <v>3.4758699999999997E-2</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D64">
+        <v>6.3209930354840389E-3</v>
+      </c>
+      <c r="E64">
+        <v>5.2860101153620201E-3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>9.2615826999999998E-3</v>
       </c>
@@ -1114,8 +1507,14 @@
       <c r="C65">
         <v>3.7927900000000001E-2</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D65">
+        <v>6.9250036181552526E-3</v>
+      </c>
+      <c r="E65">
+        <v>5.6349973573580929E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>1.0188575E-2</v>
       </c>
@@ -1125,8 +1524,14 @@
       <c r="C66">
         <v>4.12316E-2</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D66">
+        <v>7.6219944818816327E-3</v>
+      </c>
+      <c r="E66">
+        <v>6.0469996785934964E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>1.11890389E-2</v>
       </c>
@@ -1136,8 +1541,14 @@
       <c r="C67">
         <v>4.4648500000000001E-2</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D67">
+        <v>8.424008944208786E-3</v>
+      </c>
+      <c r="E67">
+        <v>6.5310010463222991E-3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>1.2338999E-2</v>
       </c>
@@ -1147,8 +1558,14 @@
       <c r="C68">
         <v>4.8158699999999999E-2</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D68">
+        <v>9.3440007191993683E-3</v>
+      </c>
+      <c r="E68">
+        <v>7.0999935476514378E-3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>1.36722007E-2</v>
       </c>
@@ -1158,8 +1575,14 @@
       <c r="C69">
         <v>5.1742999999999997E-2</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D69">
+        <v>1.0394989600037071E-2</v>
+      </c>
+      <c r="E69">
+        <v>7.7640049309068444E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>1.51778599E-2</v>
       </c>
@@ -1169,8 +1592,14 @@
       <c r="C70">
         <v>5.5383300000000003E-2</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D70">
+        <v>1.159300679723126E-2</v>
+      </c>
+      <c r="E70">
+        <v>8.5410025409203821E-3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>1.6919851400000002E-2</v>
       </c>
@@ -1180,8 +1609,14 @@
       <c r="C71">
         <v>5.9062400000000001E-2</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D71">
+        <v>1.2957997503050949E-2</v>
+      </c>
+      <c r="E71">
+        <v>9.44599660412513E-3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>1.89820531E-2</v>
       </c>
@@ -1191,8 +1626,14 @@
       <c r="C72">
         <v>6.2764200000000006E-2</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D72">
+        <v>1.4511001951534857E-2</v>
+      </c>
+      <c r="E72">
+        <v>1.0496997007656222E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>2.1319874400000001E-2</v>
       </c>
@@ -1202,8 +1643,14 @@
       <c r="C73">
         <v>6.6473199999999996E-2</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D73">
+        <v>1.6276995016087936E-2</v>
+      </c>
+      <c r="E73">
+        <v>1.171500297104134E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>2.3940661500000002E-2</v>
       </c>
@@ -1213,8 +1660,14 @@
       <c r="C74">
         <v>7.0175000000000001E-2</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D74">
+        <v>1.8283005225341403E-2</v>
+      </c>
+      <c r="E74">
+        <v>1.312199852342397E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>2.6870200600000001E-2</v>
       </c>
@@ -1224,8 +1677,14 @@
       <c r="C75">
         <v>7.3892399999999997E-2</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D75">
+        <v>2.0556994132836907E-2</v>
+      </c>
+      <c r="E75">
+        <v>1.4745005814948017E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>3.0169584199999998E-2</v>
       </c>
@@ -1235,8 +1694,14 @@
       <c r="C76">
         <v>7.7790700000000004E-2</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D76">
+        <v>2.3133006510738057E-2</v>
+      </c>
+      <c r="E76">
+        <v>1.6612994960958166E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>3.4013029899999998E-2</v>
       </c>
@@ -1246,8 +1711,14 @@
       <c r="C77">
         <v>8.2060300000000003E-2</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D77">
+        <v>2.6046000608305447E-2</v>
+      </c>
+      <c r="E77">
+        <v>1.8762003008619004E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>3.8568217000000002E-2</v>
       </c>
@@ -1257,8 +1728,14 @@
       <c r="C78">
         <v>8.6879999999999999E-2</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D78">
+        <v>2.9333995200764885E-2</v>
+      </c>
+      <c r="E78">
+        <v>2.1226992721867542E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>4.3713938700000003E-2</v>
       </c>
@@ -1268,8 +1745,14 @@
       <c r="C79">
         <v>9.2416600000000002E-2</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D79">
+        <v>3.3042001447287236E-2</v>
+      </c>
+      <c r="E79">
+        <v>2.4047000002092849E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>4.9443483000000003E-2</v>
       </c>
@@ -1279,8 +1762,14 @@
       <c r="C80">
         <v>9.8826300000000006E-2</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D80">
+        <v>3.7215004865817643E-2</v>
+      </c>
+      <c r="E80">
+        <v>2.7264003844509169E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>5.5840446299999999E-2</v>
       </c>
@@ -1290,8 +1779,14 @@
       <c r="C81">
         <v>0.1062543</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D81">
+        <v>4.1907991445499879E-2</v>
+      </c>
+      <c r="E81">
+        <v>3.0926995233830308E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>6.2805180099999997E-2</v>
       </c>
@@ -1301,8 +1796,14 @@
       <c r="C82">
         <v>0.1145014</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D82">
+        <v>4.7179010023414326E-2</v>
+      </c>
+      <c r="E82">
+        <v>3.5089008943939438E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>7.0374145799999996E-2</v>
       </c>
@@ -1312,8 +1813,14 @@
       <c r="C83">
         <v>0.1232765</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D83">
+        <v>5.3082993575798355E-2</v>
+      </c>
+      <c r="E83">
+        <v>3.9802999081742237E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>7.8849043600000002E-2</v>
       </c>
@@ -1323,8 +1830,14 @@
       <c r="C84">
         <v>0.13257939999999999</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D84">
+        <v>5.9676003847841969E-2</v>
+      </c>
+      <c r="E84">
+        <v>4.5123995605656331E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>8.8442122400000003E-2</v>
       </c>
@@ -1334,8 +1847,14 @@
       <c r="C85">
         <v>0.14241019999999999</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D85">
+        <v>6.7022002525148561E-2</v>
+      </c>
+      <c r="E85">
+        <v>5.1107997063892456E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>9.9030253200000001E-2</v>
       </c>
@@ -1345,8 +1864,14 @@
       <c r="C86">
         <v>0.15276899999999999</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D86">
+        <v>7.5194985616971091E-2</v>
+      </c>
+      <c r="E86">
+        <v>5.7818012569657698E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>0.1099420228</v>
       </c>
@@ -1356,8 +1881,14 @@
       <c r="C87">
         <v>0.16365560000000001</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D87">
+        <v>8.4275005519784493E-2</v>
+      </c>
+      <c r="E87">
+        <v>6.5317987339471875E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>0.1213510253</v>
       </c>
@@ -1367,8 +1898,14 @@
       <c r="C88">
         <v>0.17507020000000001</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D88">
+        <v>9.4338996327335722E-2</v>
+      </c>
+      <c r="E88">
+        <v>7.3677013371250308E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>0.13409527730000001</v>
       </c>
@@ -1378,8 +1915,14 @@
       <c r="C89">
         <v>0.1870127</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D89">
+        <v>0.10545000359074345</v>
+      </c>
+      <c r="E89">
+        <v>8.2968993629955287E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>0.14816282850000001</v>
       </c>
@@ -1389,8 +1932,14 @@
       <c r="C90">
         <v>0.19948299999999999</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D90">
+        <v>0.11767100219916216</v>
+      </c>
+      <c r="E90">
+        <v>9.3264991792643012E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>0.16341724439999999</v>
       </c>
@@ -1400,8 +1949,14 @@
       <c r="C91">
         <v>0.21248130000000001</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D91">
+        <v>0.13105999725466008</v>
+      </c>
+      <c r="E91">
+        <v>0.10462400136930866</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>0.17998776350000001</v>
       </c>
@@ -1411,8 +1966,14 @@
       <c r="C92">
         <v>0.2260075</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D92">
+        <v>0.14568700548414784</v>
+      </c>
+      <c r="E92">
+        <v>0.11709899626851381</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>0.19609306109999999</v>
       </c>
@@ -1422,8 +1983,14 @@
       <c r="C93">
         <v>0.24006150000000001</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D93">
+        <v>0.16167298592801504</v>
+      </c>
+      <c r="E93">
+        <v>0.13076901438242969</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>0.21009112390000001</v>
       </c>
@@ -1433,8 +2000,14 @@
       <c r="C94">
         <v>0.25464350000000002</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D94">
+        <v>0.17912701817109147</v>
+      </c>
+      <c r="E94">
+        <v>0.14571400842350557</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>0.22238837859999999</v>
       </c>
@@ -1444,8 +2017,14 @@
       <c r="C95">
         <v>0.26975339999999998</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D95">
+        <v>0.19812400491804202</v>
+      </c>
+      <c r="E95">
+        <v>0.16200298318528789</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>0.23475274730000001</v>
       </c>
@@ -1455,8 +2034,14 @@
       <c r="C96">
         <v>0.28539120000000001</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D96">
+        <v>0.21869495633986999</v>
+      </c>
+      <c r="E96">
+        <v>0.17966901211170183</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>0.24789086339999999</v>
       </c>
@@ -1466,8 +2051,14 @@
       <c r="C97">
         <v>0.30155690000000002</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D97">
+        <v>0.24082101968944433</v>
+      </c>
+      <c r="E97">
+        <v>0.19870397975605764</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>0.26205250600000002</v>
       </c>
@@ -1477,8 +2068,14 @@
       <c r="C98">
         <v>0.31825039999999999</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D98">
+        <v>0.26412804934026479</v>
+      </c>
+      <c r="E98">
+        <v>0.21899200184225354</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>0.27619663649999998</v>
       </c>
@@ -1488,8 +2085,14 @@
       <c r="C99">
         <v>0.33547189999999999</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D99">
+        <v>0.28712690624716258</v>
+      </c>
+      <c r="E99">
+        <v>0.24001896810605969</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>0.29177837350000002</v>
       </c>
@@ -1499,8 +2102,14 @@
       <c r="C100">
         <v>0.35322130000000002</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D100">
+        <v>0.30944206760727061</v>
+      </c>
+      <c r="E100">
+        <v>0.2615060111942788</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>0.30725552049999999</v>
       </c>
@@ -1510,8 +2119,14 @@
       <c r="C101">
         <v>0.37149860000000001</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D101">
+        <v>0.33107100283982765</v>
+      </c>
+      <c r="E101">
+        <v>0.28328708870766861</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>0.51639344259999997</v>
       </c>
@@ -1521,8 +2136,14 @@
       <c r="C102">
         <v>0.39030379999999998</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D102">
+        <v>0.35200105158202177</v>
+      </c>
+      <c r="E102">
+        <v>0.30520300945685119</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>0.55367231640000003</v>
       </c>
@@ -1532,8 +2153,14 @@
       <c r="C103">
         <v>0.40963699999999997</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D103">
+        <v>0.37222810437467224</v>
+      </c>
+      <c r="E103">
+        <v>0.32710382986935982</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>0.59071729959999997</v>
       </c>
@@ -1543,8 +2170,14 @@
       <c r="C104">
         <v>0.42949799999999999</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D104">
+        <v>0.39178304593171714</v>
+      </c>
+      <c r="E104">
+        <v>0.34885502759183334</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>0.6288659794</v>
       </c>
@@ -1554,8 +2187,14 @@
       <c r="C105">
         <v>0.44988689999999998</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D105">
+        <v>0.41063800379234539</v>
+      </c>
+      <c r="E105">
+        <v>0.37032598274209017</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>0.66666666669999997</v>
       </c>
@@ -1565,8 +2204,14 @@
       <c r="C106">
         <v>0.47080369999999999</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D106">
+        <v>0.42878815084079341</v>
+      </c>
+      <c r="E106">
+        <v>0.39140617661744426</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>0.66666666669999997</v>
       </c>
@@ -1576,8 +2221,14 @@
       <c r="C107">
         <v>0.49224839999999997</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D107">
+        <v>0.44623497260748513</v>
+      </c>
+      <c r="E107">
+        <v>0.41200147028063266</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>0.75</v>
       </c>
@@ -1587,8 +2238,14 @@
       <c r="C108">
         <v>0.51422109999999999</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D108">
+        <v>0.462987419197887</v>
+      </c>
+      <c r="E108">
+        <v>0.43202760202249058</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>1</v>
       </c>
@@ -1598,44 +2255,80 @@
       <c r="C109">
         <v>0.53672160000000002</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D109">
+        <v>0.47898869617740958</v>
+      </c>
+      <c r="E109">
+        <v>0.45141164952904478</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B110">
         <v>0.47082459999999998</v>
       </c>
       <c r="C110">
         <v>0.55974999999999997</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D110">
+        <v>0.49432759191785364</v>
+      </c>
+      <c r="E110">
+        <v>0.47009987031269046</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B111">
         <v>0.49339889999999997</v>
       </c>
       <c r="C111">
         <v>0.5833064</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D111">
+        <v>0.50896585605502331</v>
+      </c>
+      <c r="E111">
+        <v>0.48803497468936952</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B112">
         <v>0.51655949999999995</v>
       </c>
       <c r="C112">
         <v>0.6073906</v>
       </c>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D112">
+        <v>0.5229281307320327</v>
+      </c>
+      <c r="E112">
+        <v>0.50516853932584271</v>
+      </c>
+    </row>
+    <row r="113" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B113">
         <v>0.54030650000000002</v>
       </c>
       <c r="C113">
         <v>0.63200279999999998</v>
       </c>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D113">
+        <v>0.53617616218105557</v>
+      </c>
+      <c r="E113">
+        <v>0.52142680208075298</v>
+      </c>
+    </row>
+    <row r="114" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B114">
         <v>1</v>
       </c>
       <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114">
+        <v>1</v>
+      </c>
+      <c r="E114">
         <v>1</v>
       </c>
     </row>
@@ -1646,10 +2339,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF3D354C-BD1A-3C40-811D-4A63139399CE}">
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1659,8 +2355,14 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1670,8 +2372,14 @@
       <c r="C2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>100000</v>
       </c>
@@ -1681,9 +2389,14 @@
       <c r="C3" s="1">
         <v>100000</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D3">
+        <v>1000000</v>
+      </c>
+      <c r="E3">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>98832</v>
       </c>
@@ -1693,9 +2406,14 @@
       <c r="C4" s="1">
         <v>100000</v>
       </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D4">
+        <v>1000000</v>
+      </c>
+      <c r="E4">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>98736.0000013104</v>
       </c>
@@ -1705,9 +2423,14 @@
       <c r="C5" s="1">
         <v>100000</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D5">
+        <v>1000000</v>
+      </c>
+      <c r="E5">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>98676.999998428</v>
       </c>
@@ -1717,9 +2440,14 @@
       <c r="C6" s="1">
         <v>100000</v>
       </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <v>1000000</v>
+      </c>
+      <c r="E6">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>98630.999997898907</v>
       </c>
@@ -1729,9 +2457,14 @@
       <c r="C7" s="1">
         <v>100000</v>
       </c>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D7">
+        <v>1000000</v>
+      </c>
+      <c r="E7">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>98592.999998553307</v>
       </c>
@@ -1741,9 +2474,14 @@
       <c r="C8" s="1">
         <v>100000</v>
       </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D8">
+        <v>1000000</v>
+      </c>
+      <c r="E8">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>98558.999995458493</v>
       </c>
@@ -1753,9 +2491,14 @@
       <c r="C9" s="1">
         <v>100000</v>
       </c>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <v>1000000</v>
+      </c>
+      <c r="E9">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>98527.999996648301</v>
       </c>
@@ -1765,9 +2508,14 @@
       <c r="C10" s="1">
         <v>100000</v>
       </c>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D10">
+        <v>1000000</v>
+      </c>
+      <c r="E10">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>98498.999994236496</v>
       </c>
@@ -1777,9 +2525,14 @@
       <c r="C11" s="1">
         <v>100000</v>
       </c>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D11">
+        <v>1000000</v>
+      </c>
+      <c r="E11">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>98471.999990102602</v>
       </c>
@@ -1789,9 +2542,14 @@
       <c r="C12" s="1">
         <v>100000</v>
       </c>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D12">
+        <v>1000000</v>
+      </c>
+      <c r="E12">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>98446.999987675503</v>
       </c>
@@ -1801,9 +2559,14 @@
       <c r="C13" s="1">
         <v>100000</v>
       </c>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D13">
+        <v>1000000</v>
+      </c>
+      <c r="E13">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>98423.999992273006</v>
       </c>
@@ -1813,9 +2576,14 @@
       <c r="C14" s="1">
         <v>100000</v>
       </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D14">
+        <v>1000000</v>
+      </c>
+      <c r="E14">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>98400.999996367595</v>
       </c>
@@ -1825,9 +2593,14 @@
       <c r="C15" s="1">
         <v>100000</v>
       </c>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D15">
+        <v>1000000</v>
+      </c>
+      <c r="E15">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>98378.999992793397</v>
       </c>
@@ -1837,9 +2610,14 @@
       <c r="C16" s="1">
         <v>100000</v>
       </c>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D16">
+        <v>1000000</v>
+      </c>
+      <c r="E16">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>98353.999990180499</v>
       </c>
@@ -1849,9 +2627,14 @@
       <c r="C17" s="1">
         <v>100000</v>
       </c>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <v>1000000</v>
+      </c>
+      <c r="E17">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>98323.999994091093</v>
       </c>
@@ -1861,9 +2644,14 @@
       <c r="C18" s="1">
         <v>100000</v>
       </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <v>1000000</v>
+      </c>
+      <c r="E18">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>98285.999990215802</v>
       </c>
@@ -1873,9 +2661,14 @@
       <c r="C19" s="1">
         <v>99871.21</v>
       </c>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <v>1000000</v>
+      </c>
+      <c r="E19">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>98238.999988678697</v>
       </c>
@@ -1885,9 +2678,14 @@
       <c r="C20" s="1">
         <v>99742.476010309998</v>
       </c>
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <v>999697</v>
+      </c>
+      <c r="E20">
+        <v>999829</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>98181.999991878896</v>
       </c>
@@ -1897,9 +2695,14 @@
       <c r="C21" s="1">
         <v>99613.788267761498</v>
       </c>
-      <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <v>999387.09</v>
+      </c>
+      <c r="E21">
+        <v>999654.03</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>98118.999989763106</v>
       </c>
@@ -1909,9 +2712,14 @@
       <c r="C22" s="1">
         <v>99485.156982971297</v>
       </c>
-      <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D22">
+        <v>999069.29</v>
+      </c>
+      <c r="E22">
+        <v>999473.09</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>98054.999988134907</v>
       </c>
@@ -1921,9 +2729,14 @@
       <c r="C23" s="1">
         <v>99356.582366086499</v>
       </c>
-      <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D23">
+        <v>998742.59</v>
+      </c>
+      <c r="E23">
+        <v>999286.19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>97992.999988141397</v>
       </c>
@@ -1933,9 +2746,14 @@
       <c r="C24" s="1">
         <v>99228.054691137804</v>
       </c>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D24">
+        <v>998407.02</v>
+      </c>
+      <c r="E24">
+        <v>999092.33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>97931.999992402605</v>
       </c>
@@ -1945,9 +2763,14 @@
       <c r="C25" s="1">
         <v>99099.584128729097</v>
       </c>
-      <c r="D25" s="1"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D25">
+        <v>998060.57</v>
+      </c>
+      <c r="E25">
+        <v>998889.51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>97872.999997205596</v>
       </c>
@@ -1957,9 +2780,14 @@
       <c r="C26" s="1">
         <v>98971.170887615095</v>
       </c>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D26">
+        <v>997702.26</v>
+      </c>
+      <c r="E26">
+        <v>998676.75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>97814.9999974042</v>
       </c>
@@ -1969,9 +2797,14 @@
       <c r="C27" s="1">
         <v>98842.805278973901</v>
       </c>
-      <c r="D27" s="1"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D27">
+        <v>997329.12</v>
+      </c>
+      <c r="E27">
+        <v>998451.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>97754.999992742203</v>
       </c>
@@ -1981,9 +2814,14 @@
       <c r="C28" s="1">
         <v>98714.497433441298</v>
       </c>
-      <c r="D28" s="1"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <v>996941.16</v>
+      </c>
+      <c r="E28">
+        <v>998211.42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>97695.999991823104</v>
       </c>
@@ -1993,9 +2831,14 @@
       <c r="C29" s="1">
         <v>98586.247558375704</v>
       </c>
-      <c r="D29" s="1"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D29">
+        <v>996535.41</v>
+      </c>
+      <c r="E29">
+        <v>997955.88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>97635.999993428195</v>
       </c>
@@ -2005,8 +2848,14 @@
       <c r="C30">
         <v>98458.046002050804</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D30">
+        <v>996109.89</v>
+      </c>
+      <c r="E30">
+        <v>997680.44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>97574.999988766605</v>
       </c>
@@ -2016,8 +2865,14 @@
       <c r="C31">
         <v>98329.9028551792</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D31">
+        <v>995663.63</v>
+      </c>
+      <c r="E31">
+        <v>997383.13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>97508.999985564195</v>
       </c>
@@ -2027,8 +2882,14 @@
       <c r="C32">
         <v>98201.818323719999</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>995192.68</v>
+      </c>
+      <c r="E32">
+        <v>997060.98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>97438.999980882101</v>
       </c>
@@ -2038,8 +2899,14 @@
       <c r="C33">
         <v>98073.782792989601</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>994695.08</v>
+      </c>
+      <c r="E33">
+        <v>996710.01</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>97366.999984748007</v>
       </c>
@@ -2049,8 +2916,14 @@
       <c r="C34">
         <v>97945.727854796802</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>994167.9</v>
+      </c>
+      <c r="E34">
+        <v>996326.28</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>97289.999980139299</v>
       </c>
@@ -2060,8 +2933,14 @@
       <c r="C35">
         <v>97816.968400958795</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>993608.18</v>
+      </c>
+      <c r="E35">
+        <v>995904.83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>97207.999979265995</v>
       </c>
@@ -2071,8 +2950,14 @@
       <c r="C36">
         <v>97686.627290564604</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <v>993011.02</v>
+      </c>
+      <c r="E36">
+        <v>995440.74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>97119.999977922402</v>
       </c>
@@ -2082,8 +2967,14 @@
       <c r="C37">
         <v>97553.812552100295</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <v>992373.51</v>
+      </c>
+      <c r="E37">
+        <v>994929.09</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>97024.999981287998</v>
       </c>
@@ -2093,8 +2984,14 @@
       <c r="C38">
         <v>97417.578652871307</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>991690.76</v>
+      </c>
+      <c r="E38">
+        <v>994363.97</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>96921.999978055406</v>
       </c>
@@ -2104,8 +3001,14 @@
       <c r="C39">
         <v>97276.946636327993</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>990957.9</v>
+      </c>
+      <c r="E39">
+        <v>993738.51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>96811.999982469904</v>
       </c>
@@ -2115,8 +3018,14 @@
       <c r="C40">
         <v>97130.8950286482</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>990170.08</v>
+      </c>
+      <c r="E40">
+        <v>993046.87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>96690.999978670603</v>
       </c>
@@ -2126,8 +3035,14 @@
       <c r="C41">
         <v>96978.302392558195</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>989321.51</v>
+      </c>
+      <c r="E41">
+        <v>992281.23</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>96560.999983131202</v>
       </c>
@@ -2137,8 +3052,14 @@
       <c r="C42">
         <v>96817.948769552095</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D42">
+        <v>988406.39</v>
+      </c>
+      <c r="E42">
+        <v>991433.82</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>96418.999983703005</v>
       </c>
@@ -2148,8 +3069,14 @@
       <c r="C43">
         <v>96648.507677410598</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D43">
+        <v>987417.98</v>
+      </c>
+      <c r="E43">
+        <v>990495.93</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>96262.999981139699</v>
       </c>
@@ -2159,8 +3086,14 @@
       <c r="C44">
         <v>96468.577150667494</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D44">
+        <v>986348.61</v>
+      </c>
+      <c r="E44">
+        <v>989459.87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>96093.999984531896</v>
       </c>
@@ -2170,8 +3103,14 @@
       <c r="C45">
         <v>96276.643269568594</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D45">
+        <v>985191.62</v>
+      </c>
+      <c r="E45">
+        <v>988316.05</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>95909.999981332294</v>
       </c>
@@ -2181,8 +3120,14 @@
       <c r="C46">
         <v>96071.111891516703</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D46">
+        <v>983937.47</v>
+      </c>
+      <c r="E46">
+        <v>987055.95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>95706.999982855807</v>
       </c>
@@ -2192,8 +3137,14 @@
       <c r="C47">
         <v>95850.244405278107</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D47">
+        <v>982576.68</v>
+      </c>
+      <c r="E47">
+        <v>985670.12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>95484.999978118401</v>
       </c>
@@ -2203,8 +3154,14 @@
       <c r="C48">
         <v>95612.008622808804</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D48">
+        <v>981100.85</v>
+      </c>
+      <c r="E48">
+        <v>984148.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>95244.999977530402</v>
       </c>
@@ -2214,8 +3171,14 @@
       <c r="C49">
         <v>95354.009178741006</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D49">
+        <v>979498.72</v>
+      </c>
+      <c r="E49">
+        <v>982482.08</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>94982.999974445207</v>
       </c>
@@ -2225,8 +3188,14 @@
       <c r="C50">
         <v>95073.534896142606</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D50">
+        <v>977758.15</v>
+      </c>
+      <c r="E50">
+        <v>980660.56</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>94697.999978149106</v>
       </c>
@@ -2236,8 +3205,14 @@
       <c r="C51">
         <v>94767.521709372406</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D51">
+        <v>975868.14</v>
+      </c>
+      <c r="E51">
+        <v>978674.73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>94387.999976669496</v>
       </c>
@@ -2247,8 +3222,14 @@
       <c r="C52">
         <v>94432.632241155807</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D52">
+        <v>973815.89</v>
+      </c>
+      <c r="E52">
+        <v>976515.77</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>94055.999974787104</v>
       </c>
@@ -2258,8 +3239,14 @@
       <c r="C53">
         <v>94067.036305434201</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D53">
+        <v>971585.85</v>
+      </c>
+      <c r="E53">
+        <v>974173.11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>93701.999978030799</v>
       </c>
@@ -2269,8 +3256,14 @@
       <c r="C54">
         <v>93670.299173112406</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D54">
+        <v>969162.72</v>
+      </c>
+      <c r="E54">
+        <v>971639.28</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>93321.999978410502</v>
       </c>
@@ -2280,8 +3273,14 @@
       <c r="C55">
         <v>93241.495277557697</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D55">
+        <v>966529.5</v>
+      </c>
+      <c r="E55">
+        <v>968906.06</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>92909.999978486201</v>
       </c>
@@ -2291,8 +3290,14 @@
       <c r="C56">
         <v>92779.241240569696</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D56">
+        <v>963668.57</v>
+      </c>
+      <c r="E56">
+        <v>965967.37</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>92464.999980006294</v>
       </c>
@@ -2302,8 +3307,14 @@
       <c r="C57">
         <v>92281.703281492999</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D57">
+        <v>960560.74</v>
+      </c>
+      <c r="E57">
+        <v>962816.38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>91986.999980435605</v>
       </c>
@@ -2313,8 +3324,14 @@
       <c r="C58">
         <v>91746.607825015293</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D58">
+        <v>957187.25</v>
+      </c>
+      <c r="E58">
+        <v>959449.42</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>91477.9999794217</v>
       </c>
@@ -2324,8 +3341,14 @@
       <c r="C59">
         <v>91171.283196666205</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D59">
+        <v>953527.93</v>
+      </c>
+      <c r="E59">
+        <v>955862.03</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>90937.999975784594</v>
       </c>
@@ -2335,8 +3358,14 @@
       <c r="C60">
         <v>90552.676923048493</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D60">
+        <v>949562.2</v>
+      </c>
+      <c r="E60">
+        <v>952053.88</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>90363.999974691003</v>
       </c>
@@ -2346,8 +3375,14 @@
       <c r="C61">
         <v>89887.386405694895</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D61">
+        <v>945267.33</v>
+      </c>
+      <c r="E61">
+        <v>948023.84</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>89753.999970634293</v>
       </c>
@@ -2357,8 +3392,14 @@
       <c r="C62">
         <v>89171.694046394099</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D62">
+        <v>940621.35</v>
+      </c>
+      <c r="E62">
+        <v>943772.9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>89105.999974385704</v>
       </c>
@@ -2368,8 +3409,14 @@
       <c r="C63">
         <v>88401.598379439994</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D63">
+        <v>935600.31</v>
+      </c>
+      <c r="E63">
+        <v>939304.13</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>88416.999974731501</v>
       </c>
@@ -2379,8 +3426,14 @@
       <c r="C64">
         <v>87572.886435591805</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D64">
+        <v>930176.63</v>
+      </c>
+      <c r="E64">
+        <v>934616.07</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>87673.999978881795</v>
       </c>
@@ -2390,8 +3443,14 @@
       <c r="C65">
         <v>86681.1492475954</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D65">
+        <v>924296.99</v>
+      </c>
+      <c r="E65">
+        <v>929675.68</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>86861.999977437605</v>
       </c>
@@ -2401,8 +3460,14 @@
       <c r="C66">
         <v>85721.866305102099</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D66">
+        <v>917896.23</v>
+      </c>
+      <c r="E66">
+        <v>924436.96</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>85976.999976017396</v>
       </c>
@@ -2412,8 +3477,14 @@
       <c r="C67">
         <v>84696.812800012398</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D67">
+        <v>910900.03</v>
+      </c>
+      <c r="E67">
+        <v>918846.89</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>85014.999978780499</v>
       </c>
@@ -2423,8 +3494,14 @@
       <c r="C68">
         <v>83611.160583860503</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D68">
+        <v>903226.6</v>
+      </c>
+      <c r="E68">
+        <v>912845.9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>83965.999979057306</v>
       </c>
@@ -2434,8 +3511,14 @@
       <c r="C69">
         <v>82465.963600691597</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D69">
+        <v>894786.85</v>
+      </c>
+      <c r="E69">
+        <v>906364.7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>82817.999975367406</v>
       </c>
@@ -2445,8 +3528,14 @@
       <c r="C70">
         <v>81258.661893577402</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D70">
+        <v>885485.55</v>
+      </c>
+      <c r="E70">
+        <v>899327.68</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>81560.999974543098</v>
       </c>
@@ -2456,8 +3545,14 @@
       <c r="C71">
         <v>79983.607852206798</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D71">
+        <v>875220.11</v>
+      </c>
+      <c r="E71">
+        <v>891646.52</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>80180.999974938401</v>
       </c>
@@ -2467,8 +3562,14 @@
       <c r="C72">
         <v>78632.588735253594</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D72">
+        <v>863879.01</v>
+      </c>
+      <c r="E72">
+        <v>883224.03</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>78658.999975803104</v>
       </c>
@@ -2478,8 +3579,14 @@
       <c r="C73">
         <v>77195.373731386106</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D73">
+        <v>851343.26</v>
+      </c>
+      <c r="E73">
+        <v>873952.83</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>76981.999975889295</v>
       </c>
@@ -2489,8 +3596,14 @@
       <c r="C74">
         <v>75660.258809826395</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D74">
+        <v>837485.95</v>
+      </c>
+      <c r="E74">
+        <v>863714.47</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>75138.9999728736</v>
       </c>
@@ -2500,8 +3613,14 @@
       <c r="C75">
         <v>74014.678444816207</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D75">
+        <v>822174.19</v>
+      </c>
+      <c r="E75">
+        <v>852380.81</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>73119.999970719</v>
       </c>
@@ -2511,8 +3630,14 @@
       <c r="C76">
         <v>72246.526988512298</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D76">
+        <v>805272.76</v>
+      </c>
+      <c r="E76">
+        <v>839812.45</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>70913.999974898397</v>
       </c>
@@ -2522,8 +3647,14 @@
       <c r="C77">
         <v>70347.433106134107</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D77">
+        <v>786644.38</v>
+      </c>
+      <c r="E77">
+        <v>825860.65</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>68501.999973423604</v>
       </c>
@@ -2533,8 +3664,14 @@
       <c r="C78">
         <v>68313.414460046697</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D78">
+        <v>766155.44</v>
+      </c>
+      <c r="E78">
+        <v>810365.85</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>65859.999973514598</v>
       </c>
@@ -2544,8 +3681,14 @@
       <c r="C79">
         <v>66144.723141915194</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D79">
+        <v>743681.04</v>
+      </c>
+      <c r="E79">
+        <v>793164.22</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>62980.9999718904</v>
       </c>
@@ -2555,8 +3698,14 @@
       <c r="C80">
         <v>63845.6185536423</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D80">
+        <v>719108.33</v>
+      </c>
+      <c r="E80">
+        <v>774091</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>59866.999970457196</v>
       </c>
@@ -2566,8 +3715,14 @@
       <c r="C81">
         <v>61424.0883177016</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D81">
+        <v>692346.71</v>
+      </c>
+      <c r="E81">
+        <v>752986.18</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>56523.999973464801</v>
       </c>
@@ -2577,8 +3732,14 @@
       <c r="C82">
         <v>58891.474877821398</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D82">
+        <v>663331.85</v>
+      </c>
+      <c r="E82">
+        <v>729698.58</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>52973.999975158898</v>
       </c>
@@ -2588,8 +3749,14 @@
       <c r="C83">
         <v>56262.058861739002</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D83">
+        <v>632036.51</v>
+      </c>
+      <c r="E83">
+        <v>704094.18</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>49245.999977297899</v>
       </c>
@@ -2599,8 +3766,14 @@
       <c r="C84">
         <v>53552.551247634197</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D84">
+        <v>598486.12</v>
+      </c>
+      <c r="E84">
+        <v>676069.12</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>45362.999977962303</v>
       </c>
@@ -2610,8 +3783,14 @@
       <c r="C85">
         <v>50781.581588427798</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D85">
+        <v>562770.86</v>
+      </c>
+      <c r="E85">
+        <v>645562.18000000005</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>41350.999981480199</v>
       </c>
@@ -2621,8 +3800,14 @@
       <c r="C86">
         <v>47969.130020841498</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D86">
+        <v>525052.82999999996</v>
+      </c>
+      <c r="E86">
+        <v>612568.79</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>37255.999983241003</v>
       </c>
@@ -2632,8 +3817,14 @@
       <c r="C87">
         <v>45135.958075898503</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D87">
+        <v>485571.49</v>
+      </c>
+      <c r="E87">
+        <v>577151.28</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>33159.999983646703</v>
       </c>
@@ -2643,8 +3834,14 @@
       <c r="C88">
         <v>42303.035776031204</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D88">
+        <v>444649.95</v>
+      </c>
+      <c r="E88">
+        <v>539452.92000000004</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>29135.9999866832</v>
       </c>
@@ -2654,8 +3851,14 @@
       <c r="C89">
         <v>39491.017618283899</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D89">
+        <v>402702.12</v>
+      </c>
+      <c r="E89">
+        <v>499707.64</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>25228.999989056101</v>
       </c>
@@ -2665,8 +3868,14 @@
       <c r="C90">
         <v>36719.735456920796</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D90">
+        <v>360237.18</v>
+      </c>
+      <c r="E90">
+        <v>458247.4</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>21490.999990451099</v>
       </c>
@@ -2676,8 +3885,14 @@
       <c r="C91">
         <v>34006.426076643897</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D91">
+        <v>317847.71000000002</v>
+      </c>
+      <c r="E91">
+        <v>415508.96</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>17978.999992611101</v>
       </c>
@@ -2687,8 +3902,14 @@
       <c r="C92">
         <v>31361.042387643502</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D92">
+        <v>276190.59000000003</v>
+      </c>
+      <c r="E92">
+        <v>372036.75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>14742.999993974499</v>
       </c>
@@ -2698,8 +3919,14 @@
       <c r="C93">
         <v>28787.545841000701</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D93">
+        <v>235953.21</v>
+      </c>
+      <c r="E93">
+        <v>328471.62</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>11851.999995358799</v>
       </c>
@@ -2709,8 +3936,14 @@
       <c r="C94">
         <v>26286.483858334599</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D94">
+        <v>197805.95</v>
+      </c>
+      <c r="E94">
+        <v>285517.71000000002</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>9361.9999958710905</v>
       </c>
@@ -2720,8 +3953,14 @@
       <c r="C95">
         <v>23857.1763941924</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D95">
+        <v>162373.56</v>
+      </c>
+      <c r="E95">
+        <v>243913.78</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>7279.9999963361097</v>
       </c>
@@ -2731,8 +3970,14 @@
       <c r="C96">
         <v>21499.459922706999</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D96">
+        <v>130203.46</v>
+      </c>
+      <c r="E96">
+        <v>204399.02</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>5570.9999968522197</v>
       </c>
@@ -2742,8 +3987,14 @@
       <c r="C97">
         <v>19215.049858241699</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D97">
+        <v>101728.62</v>
+      </c>
+      <c r="E97">
+        <v>167674.85</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>4189.9999976311201</v>
       </c>
@@ -2753,8 +4004,14 @@
       <c r="C98">
         <v>17014.899748403299</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D98">
+        <v>77230.23</v>
+      </c>
+      <c r="E98">
+        <v>134357.19</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>3091.9999981118899</v>
       </c>
@@ -2764,8 +4021,14 @@
       <c r="C99">
         <v>14917.3624595692</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D99">
+        <v>56831.56</v>
+      </c>
+      <c r="E99">
+        <v>104934.04</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>2237.9999985753798</v>
       </c>
@@ -2775,8 +4038,14 @@
       <c r="C100">
         <v>12939.627495097</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D100">
+        <v>40513.69</v>
+      </c>
+      <c r="E100">
+        <v>79747.88</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>1584.99999909805</v>
       </c>
@@ -2786,8 +4055,14 @@
       <c r="C101">
         <v>11096.892555594701</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D101">
+        <v>27977.05</v>
+      </c>
+      <c r="E101">
+        <v>58893.33</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>1097.99999938268</v>
       </c>
@@ -2797,8 +4072,14 @@
       <c r="C102">
         <v>9401.6313767691099</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D102">
+        <v>18714.66</v>
+      </c>
+      <c r="E102">
+        <v>42209.61</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>530.99999972666103</v>
       </c>
@@ -2808,8 +4089,14 @@
       <c r="C103">
         <v>7863.0017528251401</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D103">
+        <v>12127.08</v>
+      </c>
+      <c r="E103">
+        <v>29327.11</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>236.999999869601</v>
       </c>
@@ -2819,8 +4106,14 @@
       <c r="C104">
         <v>6486.42446335769</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D104">
+        <v>7613.04</v>
+      </c>
+      <c r="E104">
+        <v>19734.099999999999</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>96.999999941430104</v>
       </c>
@@ -2830,8 +4123,14 @@
       <c r="C105">
         <v>5273.38071111912</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D105">
+        <v>4630.38</v>
+      </c>
+      <c r="E105">
+        <v>12849.76</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>35.999999976462703</v>
       </c>
@@ -2841,8 +4140,14 @@
       <c r="C106">
         <v>4221.4309067229397</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D106">
+        <v>2728.97</v>
+      </c>
+      <c r="E106">
+        <v>8091.16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>11.999999990954199</v>
       </c>
@@ -2852,8 +4157,14 @@
       <c r="C107">
         <v>3324.4557798022702</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D107">
+        <v>1558.82</v>
+      </c>
+      <c r="E107">
+        <v>4924.2299999999996</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>3.9999999965847501</v>
       </c>
@@ -2863,8 +4174,14 @@
       <c r="C108">
         <v>2573.1038401486098</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D108">
+        <v>863.22</v>
+      </c>
+      <c r="E108">
+        <v>2895.44</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>0.99999999914618698</v>
       </c>
@@ -2874,8 +4191,14 @@
       <c r="C109">
         <v>1955.4006726267701</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D109">
+        <v>463.56</v>
+      </c>
+      <c r="E109">
+        <v>1644.53</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>0</v>
       </c>
@@ -2885,48 +4208,84 @@
       <c r="C110">
         <v>1457.4706014467299</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D110">
+        <v>241.52</v>
+      </c>
+      <c r="E110">
+        <v>902.17</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B111">
         <v>5795.1718490413996</v>
       </c>
       <c r="C111">
         <v>1064.31295130643</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D111">
+        <v>122.13</v>
+      </c>
+      <c r="E111">
+        <v>478.06</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B112">
         <v>4541.39105563877</v>
       </c>
       <c r="C112">
         <v>760.56740095755094</v>
       </c>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D112">
+        <v>59.97</v>
+      </c>
+      <c r="E112">
+        <v>244.75</v>
+      </c>
+    </row>
+    <row r="113" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B113">
         <v>3493.6249265152801</v>
       </c>
       <c r="C113">
         <v>531.21305328373501</v>
       </c>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D113">
+        <v>28.61</v>
+      </c>
+      <c r="E113">
+        <v>121.11</v>
+      </c>
+    </row>
+    <row r="114" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B114">
         <v>2635.3572704180301</v>
       </c>
       <c r="C114">
         <v>362.154286590965</v>
       </c>
-    </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D114">
+        <v>13.27</v>
+      </c>
+      <c r="E114">
+        <v>57.96</v>
+      </c>
+    </row>
+    <row r="115" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B115">
         <v>1946.9885110627599</v>
       </c>
       <c r="C115">
         <v>240.66169997514899</v>
       </c>
-    </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D115">
+        <v>0</v>
+      </c>
+      <c r="E115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B116">
         <v>1407.0307713862801</v>
       </c>
@@ -2934,7 +4293,7 @@
         <v>155.654861449717</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B117">
         <v>993.30645844632102</v>
       </c>
@@ -2942,7 +4301,7 @@
         <v>97.829298337953304</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B118">
         <v>684.05241228655996</v>
       </c>
@@ -2950,7 +4309,7 @@
         <v>59.646151445316399</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B119">
         <v>458.847514224478</v>
       </c>
@@ -2958,7 +4317,7 @@
         <v>35.212880905711302</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B120">
         <v>299.31008784774599</v>
       </c>
@@ -2966,7 +4325,7 @@
         <v>20.089018982470101</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B121">
         <v>189.53871174976101</v>
       </c>
@@ -2974,7 +4333,7 @@
         <v>11.0512325084054</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B122">
         <v>116.302735193543</v>
       </c>
@@ -2982,7 +4341,7 @@
         <v>5.8482713538878999</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B123">
         <v>69.011763530239094</v>
       </c>
@@ -2990,7 +4349,7 @@
         <v>2.96946913717075</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B124">
         <v>39.513727286867699</v>
       </c>
@@ -2998,7 +4357,7 @@
         <v>1.4425054510387501</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B125">
         <v>21.7785202781028</v>
       </c>
@@ -3006,7 +4365,7 @@
         <v>0.66828161734851299</v>
       </c>
     </row>
-    <row r="126" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B126">
         <v>11.524657179573101</v>
       </c>
@@ -3014,7 +4373,7 @@
         <v>0.29421098203768298</v>
       </c>
     </row>
-    <row r="127" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B127">
         <v>5.8384040042946603</v>
       </c>
@@ -3022,7 +4381,7 @@
         <v>0.122595833264817</v>
       </c>
     </row>
-    <row r="128" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B128">
         <v>2.8225209510382099</v>
       </c>

</xml_diff>